<commit_message>
v5H226z108n12: BAT 좀비 자동 청소 + KNK_중지.bat 추가
- KNK_시작.bat / START.bat 기동 직전 PowerShell 한줄로:
  1) 8081 포트 점유 PID 강제 종료
  2) parent_pid 죽은 spawn_main 좀비 워커 청소
- KNK_중지.bat 신설 (수동 실행용, 동일 로직 + 진행 로그)
- uvicorn reload=True 의 Windows orphan 워커 재발 방지
</commit_message>
<xml_diff>
--- a/KNK업무시스템구축/참고자료/형태별업무진행순서.xlsx
+++ b/KNK업무시스템구축/참고자료/형태별업무진행순서.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\top00\JR\Claude 코드\KNK업무시스템구축\참고자료\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF085724-4874-4472-BE99-724984F8CC6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{665CAC47-99DE-43B9-BBA0-7E8C7D50E3AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="34452" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{064EE91B-9D61-4F10-B9D7-767966E129AA}"/>
+    <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="21840" xr2:uid="{064EE91B-9D61-4F10-B9D7-767966E129AA}"/>
   </bookViews>
   <sheets>
     <sheet name="본사PO" sheetId="1" r:id="rId1"/>

</xml_diff>